<commit_message>
MACE neural-potential runner: CPU/GPU one-click for Windows and Linux
- scripts/run_main_mace.py: NPT runner (FePt_potential.pt, auto/cpu/cuda
  with cuda->cpu fallback, own .lmp parser, CTE report)
- run_mace.bat + run_lammps.sh: one-click launchers (auto-bootstrap venv
  on first run)
- bootstrap_mace.bat/sh, bootstrap_lammps.sh: one-time env setup
  (torch 2.11 cu128 + requirements-mace.txt, apt lammps on Linux)
- requirements-mace.txt: pinned MACE pipeline dependencies
- lmp_helper.py: gen_structure now fails loudly on subprocess errors
- make_release.bat/sh: Windows zip + Linux tar.gz release builders
- potentials/FePt_potential.pt + Zhou04.eam.alloy now tracked in git
- .gitignore: .venv-mace/, output_mace_*/, *.tar.gz, *.bak_hermes*
- README: MACE section (Windows/Linux, CPU/GPU usage)
</commit_message>
<xml_diff>
--- a/output_v4_256/all_results_turbo_256at_omp.xlsx
+++ b/output_v4_256/all_results_turbo_256at_omp.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +458,7 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,13 +536,13 @@
         <v>300</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3.627013</v>
+        <v>3.627059</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.004484</v>
+        <v>0.003577</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.000206745283375831</v>
+        <v>0.0004831584405944334</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>302</v>
@@ -554,7 +554,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>742.37</v>
+        <v>869.97</v>
       </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         <v>100000</v>
       </c>
       <c r="M2" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="3">
@@ -579,13 +579,13 @@
         <v>500</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3.637386</v>
+        <v>3.637431</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.004471</v>
+        <v>0.004049</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>5.791148444922456e-05</v>
+        <v>0.0007337167559038349</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>302</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>758.45</v>
+        <v>891.8</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
@@ -611,7 +611,7 @@
         <v>100000</v>
       </c>
       <c r="M3" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="4">
@@ -622,13 +622,13 @@
         <v>700</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3.647557</v>
+        <v>3.647623</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.007162</v>
+        <v>0.007204</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.001052798034361313</v>
+        <v>0.0009405852748658461</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>302</v>
@@ -640,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>762.64</v>
+        <v>898.0599999999999</v>
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         <v>100000</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="5">
@@ -665,13 +665,13 @@
         <v>900</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3.658476</v>
+        <v>3.658307</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.00699</v>
+        <v>0.007825</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.001384109686676904</v>
+        <v>0.001078471311693363</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>302</v>
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>764.51</v>
+        <v>898.62</v>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v>100000</v>
       </c>
       <c r="M5" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="6">
@@ -708,13 +708,13 @@
         <v>1100</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3.669001</v>
+        <v>3.668816</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.008758999999999999</v>
+        <v>0.009315</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.001230467103037647</v>
+        <v>0.0006965142304871108</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>302</v>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>762.89</v>
+        <v>897.26</v>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
         <v>100000</v>
       </c>
       <c r="M6" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="7">
@@ -751,13 +751,13 @@
         <v>1200</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3.674681</v>
+        <v>3.674294</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.009625999999999999</v>
+        <v>0.008538</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.002168316447893837</v>
+        <v>0.002103488827125854</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>302</v>
@@ -769,7 +769,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>762.55</v>
+        <v>896.83</v>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         <v>100000</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="8">
@@ -794,25 +794,25 @@
         <v>300</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3.797485</v>
+        <v>7.591374</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.002919</v>
+        <v>0.001919</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0001175205198964413</v>
+        <v>-4.823141888987692e-05</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>219</v>
+        <v>9.4</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>5308.7</v>
+        <v>1772.4</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>600.38</v>
+        <v>5111.31</v>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>100000</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="9">
@@ -837,25 +837,25 @@
         <v>500</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3.806623</v>
+        <v>7.60616</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.003913</v>
+        <v>0.002332</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.001911971668510759</v>
+        <v>-0.000425684679711047</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-38.1</v>
+        <v>107.6</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>6725.7</v>
+        <v>2039.3</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>597.9400000000001</v>
+        <v>5067.12</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -869,7 +869,7 @@
         <v>100000</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="10">
@@ -880,25 +880,25 @@
         <v>700</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3.814489</v>
+        <v>7.619431</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0.004132</v>
+        <v>0.003003</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0001644838124441605</v>
+        <v>1.088000339333206e-05</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>14.1</v>
+        <v>-39.3</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>7154.6</v>
+        <v>2699.6</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>593.88</v>
+        <v>5070.03</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
         <v>100000</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="11">
@@ -923,25 +923,25 @@
         <v>900</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3.821398</v>
+        <v>7.6328</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.00562</v>
+        <v>0.003616</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.0003760983323730649</v>
+        <v>-6.352522061003896e-05</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>93.59999999999999</v>
+        <v>114.1</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>9288.1</v>
+        <v>3054.7</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>591.53</v>
+        <v>5039.84</v>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         <v>100000</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1100</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3.828275</v>
+        <v>7.6481</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.005651</v>
+        <v>0.004196</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0001296687804255292</v>
+        <v>0.0002165462404857266</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>378.1</v>
+        <v>120.1</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>9288.299999999999</v>
+        <v>3400.8</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>598.25</v>
+        <v>5021.98</v>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         <v>100000</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="13">
@@ -1009,25 +1009,25 @@
         <v>1200</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3.831604</v>
+        <v>7.654133</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.006622</v>
+        <v>0.004203</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.0008327208929994612</v>
+        <v>-3.725804605281269e-06</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-296.3</v>
+        <v>28</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>10970.3</v>
+        <v>3455.2</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>595.97</v>
+        <v>5012.19</v>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>100000</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="14">
@@ -1052,25 +1052,25 @@
         <v>300</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>3.869811</v>
+        <v>3.869815</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.002398</v>
+        <v>0.002303</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.00018721428144719</v>
+        <v>0.0001507986065241163</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12.3</v>
+        <v>36.9</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>5275.9</v>
+        <v>4855</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>541.12</v>
+        <v>632.72</v>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         <v>100000</v>
       </c>
       <c r="M14" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="15">
@@ -1095,25 +1095,25 @@
         <v>500</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>3.875957</v>
+        <v>3.875782</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.003285</v>
+        <v>0.003117</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>2.815560017443985e-05</v>
+        <v>6.47313857342624e-05</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>-7.2</v>
+        <v>-180.6</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>6994.8</v>
+        <v>6744.4</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>541.01</v>
+        <v>636.5700000000001</v>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
         <v>100000</v>
       </c>
       <c r="M15" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="16">
@@ -1138,25 +1138,25 @@
         <v>700</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>3.881715</v>
+        <v>3.881446</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.003549</v>
+        <v>0.004182</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0001709884694141017</v>
+        <v>-0.0002988878511622772</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>-19.8</v>
+        <v>365.3</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>7584.1</v>
+        <v>8835.6</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>547.21</v>
+        <v>634.96</v>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         <v>100000</v>
       </c>
       <c r="M16" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="17">
@@ -1181,25 +1181,25 @@
         <v>900</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>3.887403</v>
+        <v>3.887491</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.004692</v>
+        <v>0.004548</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.0001006077217908796</v>
+        <v>-0.0001581840780930932</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-67.8</v>
+        <v>429.9</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>9464.299999999999</v>
+        <v>9092.5</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>546.27</v>
+        <v>631.02</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         <v>100000</v>
       </c>
       <c r="M17" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="18">
@@ -1224,25 +1224,25 @@
         <v>1100</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>3.892813</v>
+        <v>3.892837</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.004747</v>
+        <v>0.005168</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.0005830894567528944</v>
+        <v>-7.688552990270381e-06</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>230.3</v>
+        <v>-302.7</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>9760.799999999999</v>
+        <v>10116.6</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>543.14</v>
+        <v>576.35</v>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
         <v>100000</v>
       </c>
       <c r="M18" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="19">
@@ -1267,25 +1267,25 @@
         <v>1200</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>3.895203</v>
+        <v>3.895584</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.005784</v>
+        <v>0.005046</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.0003641679767212302</v>
+        <v>0.0004804726056217845</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>112.3</v>
+        <v>-79.3</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>11756.5</v>
+        <v>10047.2</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>542.37</v>
+        <v>573.92</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>100000</v>
       </c>
       <c r="M19" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="20">
@@ -1310,25 +1310,25 @@
         <v>300</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>3.905901</v>
+        <v>3.905928</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0.002374</v>
+        <v>0.002322</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.0001764662036540798</v>
+        <v>0.0001044443743585255</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>12</v>
+        <v>-41</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>5458.5</v>
+        <v>5204.7</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>470.26</v>
+        <v>504.4</v>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>100000</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="21">
@@ -1353,25 +1353,25 @@
         <v>500</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>3.911772</v>
+        <v>3.911848</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.003014</v>
+        <v>0.00298</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.0001077015538459847</v>
+        <v>9.250582834186005e-05</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>54.7</v>
+        <v>94.3</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>6766</v>
+        <v>6399.7</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>480.74</v>
+        <v>513.51</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
         <v>100000</v>
       </c>
       <c r="M21" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="22">
@@ -1396,25 +1396,25 @@
         <v>700</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>3.917635</v>
+        <v>3.917472</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0.003548</v>
+        <v>0.003479</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.0001994024270857153</v>
+        <v>0.0002149200655732209</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>-26</v>
+        <v>139.3</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>8055.3</v>
+        <v>7556.7</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>459.36</v>
+        <v>593.74</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -1428,7 +1428,7 @@
         <v>100000</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="23">
@@ -1439,25 +1439,25 @@
         <v>900</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3.922835</v>
+        <v>3.9229</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.004197</v>
+        <v>0.004225</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.0001352300883885604</v>
+        <v>0.0003333960605802488</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>228.7</v>
+        <v>-13</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>8913.299999999999</v>
+        <v>9013.6</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>459.36</v>
+        <v>598.4</v>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         <v>100000</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="24">
@@ -1482,25 +1482,25 @@
         <v>1100</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>3.927883</v>
+        <v>3.928096</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0.004543</v>
+        <v>0.005056</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-6.349602578925584e-05</v>
+        <v>-0.0001180152811683932</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>-18.2</v>
+        <v>-210.7</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>9454.4</v>
+        <v>10321.8</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>449.52</v>
+        <v>616.7</v>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         <v>100000</v>
       </c>
       <c r="M24" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="25">
@@ -1525,25 +1525,25 @@
         <v>1200</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>3.930933</v>
+        <v>3.930677</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0.005158</v>
+        <v>0.004857</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.0001783910921084875</v>
+        <v>0.0003778122312589893</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>18.8</v>
+        <v>146.7</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>11255.6</v>
+        <v>10061.1</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>448.57</v>
+        <v>617.1799999999999</v>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         <v>100000</v>
       </c>
       <c r="M25" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="26">
@@ -1568,25 +1568,25 @@
         <v>300</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>3.929026</v>
+        <v>3.928964</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0.002334</v>
+        <v>0.002396</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0002069683753966878</v>
+        <v>-0.0001071383928561431</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>33.7</v>
+        <v>-12.4</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>4902.6</v>
+        <v>5026.8</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>141.32</v>
+        <v>187.71</v>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
         <v>100000</v>
       </c>
       <c r="M26" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="27">
@@ -1611,25 +1611,25 @@
         <v>500</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>3.935243</v>
+        <v>3.935331</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0.003046</v>
+        <v>0.002954</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>2.326997710211387e-05</v>
+        <v>-0.0001637527173947717</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>-0.9</v>
+        <v>3.3</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>6204.3</v>
+        <v>6022.6</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>140.28</v>
+        <v>185.9</v>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         <v>100000</v>
       </c>
       <c r="M27" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="28">
@@ -1654,25 +1654,25 @@
         <v>700</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>3.94211</v>
+        <v>3.942225</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0.003848</v>
+        <v>0.003701</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-0.0004160894334233056</v>
+        <v>-0.0005068907666179179</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>108.7</v>
+        <v>-115.7</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>7531.2</v>
+        <v>7320.5</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>137.49</v>
+        <v>183.6</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
         <v>100000</v>
       </c>
       <c r="M28" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="29">
@@ -1697,25 +1697,25 @@
         <v>900</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3.94933</v>
+        <v>3.949583</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.004194</v>
+        <v>0.004217</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.0001332570078940165</v>
+        <v>-0.0006408853124244551</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>-76.3</v>
+        <v>102.1</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>8051.5</v>
+        <v>8141.8</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>135.39</v>
+        <v>183.65</v>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
@@ -1729,7 +1729,7 @@
         <v>100000</v>
       </c>
       <c r="M29" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="30">
@@ -1740,25 +1740,25 @@
         <v>1100</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3.957704</v>
+        <v>3.957531</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>0.004926</v>
+        <v>0.004886</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>5.981112428887769e-06</v>
+        <v>8.947753506349798e-05</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>-91.59999999999999</v>
+        <v>-234.8</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>9164.9</v>
+        <v>9127.6</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>135.08</v>
+        <v>189.83</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -1772,7 +1772,7 @@
         <v>100000</v>
       </c>
       <c r="M30" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
     <row r="31">
@@ -1783,25 +1783,25 @@
         <v>1200</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>3.961384</v>
+        <v>3.961072</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.00563</v>
+        <v>0.005501</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-0.0003303789607249641</v>
+        <v>-0.0004427870346903617</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>202</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>56.2</v>
+        <v>42.7</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>10355.7</v>
+        <v>9933.299999999999</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>135.14</v>
+        <v>191.54</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
         <v>100000</v>
       </c>
       <c r="M31" s="8" t="n">
-        <v>26365</v>
+        <v>123321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>